<commit_message>
17.08.2026 - zwrot produkty, dogrywanie progressbar per rama & wgrywanie receptur zapis
</commit_message>
<xml_diff>
--- a/Produkty/014-50076014.xlsx
+++ b/Produkty/014-50076014.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -563,132 +563,9 @@
         <v/>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v/>
-      </c>
-      <c r="B5" t="str">
-        <v>250x60x28</v>
-      </c>
-      <c r="C5" t="str">
-        <v>250</v>
-      </c>
-      <c r="D5" t="str">
-        <v>28</v>
-      </c>
-      <c r="E5" t="str">
-        <v>60</v>
-      </c>
-      <c r="F5" t="str">
-        <v>BUK</v>
-      </c>
-      <c r="G5" t="str">
-        <v>1</v>
-      </c>
-      <c r="H5" t="str">
-        <v>1</v>
-      </c>
-      <c r="I5" t="str">
-        <v>1</v>
-      </c>
-      <c r="J5" t="str">
-        <v>1</v>
-      </c>
-      <c r="K5" t="str">
-        <v>1</v>
-      </c>
-      <c r="L5" t="str">
-        <v/>
-      </c>
-      <c r="M5" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v/>
-      </c>
-      <c r="B6" t="str">
-        <v>300x80x28</v>
-      </c>
-      <c r="C6" t="str">
-        <v>300</v>
-      </c>
-      <c r="D6" t="str">
-        <v>28</v>
-      </c>
-      <c r="E6" t="str">
-        <v>80</v>
-      </c>
-      <c r="F6" t="str">
-        <v>BUK</v>
-      </c>
-      <c r="G6" t="str">
-        <v>2</v>
-      </c>
-      <c r="H6" t="str">
-        <v>1</v>
-      </c>
-      <c r="I6" t="str">
-        <v>1</v>
-      </c>
-      <c r="J6" t="str">
-        <v>1</v>
-      </c>
-      <c r="K6" t="str">
-        <v>2</v>
-      </c>
-      <c r="L6" t="str">
-        <v/>
-      </c>
-      <c r="M6" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v/>
-      </c>
-      <c r="B7" t="str">
-        <v>1280x32x28</v>
-      </c>
-      <c r="C7" t="str">
-        <v>1280</v>
-      </c>
-      <c r="D7" t="str">
-        <v>28</v>
-      </c>
-      <c r="E7" t="str">
-        <v>32</v>
-      </c>
-      <c r="F7" t="str">
-        <v>BUK</v>
-      </c>
-      <c r="G7" t="str">
-        <v/>
-      </c>
-      <c r="H7" t="str">
-        <v>5 i 6</v>
-      </c>
-      <c r="I7" t="str">
-        <v>2</v>
-      </c>
-      <c r="J7" t="str">
-        <v/>
-      </c>
-      <c r="K7" t="str">
-        <v>1</v>
-      </c>
-      <c r="L7" t="str">
-        <v/>
-      </c>
-      <c r="M7" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>